<commit_message>
Aggiorna checklist: password minima fatta, email conferma verificata
L'email di conferma al cliente funziona (prova reale del 01/09) ma finisce
in spam: SPF/DKIM/DMARC sono corretti, la causa e' la reputazione del
dominio, nato il 26/08. Email migliorata con versione testo, Reply-To e
firma aziendale.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CHECKLIST.xlsx
+++ b/CHECKLIST.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limitazioni note" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Da provare tu'!$A$4:$D$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Confronto CGI'!$A$4:$E$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Limitazioni note'!$A$4:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Limitazioni note'!$A$4:$D$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -542,7 +542,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Aggiornato al 31 agosto 2026. Usa i menu a tendina nelle colonne Priorita' e Stato per aggiornare la checklist.</t>
+          <t>Aggiornato al 1 settembre 2026. Usa i menu a tendina nelle colonne Priorita' e Stato per aggiornare la checklist.</t>
         </is>
       </c>
     </row>
@@ -689,17 +689,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Vortix / Lead</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Alzare la lunghezza minima password su Supabase</t>
+          <t>L'email di conferma al cliente finisce nello spam</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Il minimo predefinito e' 6 caratteri. Nei moduli chiediamo 8, ma quel controllo avviene nel browser ed e' aggirabile: quello del pannello e' applicato dal server.</t>
+          <t>Il cliente riceve la conferma nella cartella spam invece che in posta in arrivo. Rischio concreto: molti non la vedono e pensano che la richiesta non sia arrivata.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -707,9 +707,9 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>In corso</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -719,12 +719,12 @@
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Michele</t>
+          <t>Michele + Claude</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Pannello Supabase &gt; Authentication &gt; Sign In / Providers &gt; Email &gt; Minimum password length + Password Requirements. Consigliato: 8+ con numeri e lettere.</t>
+          <t>01/09: verificato che SPF, DKIM, DMARC e percorso di ritorno sono TUTTI corretti. La causa e' la reputazione: il dominio e' nato il 26/08 e non ha ancora storico di invio. Migliorata l'email (versione testo, Reply-To, firma aziendale). AZIONE PER TE: apri l'email nello spam e premi 'Segnala come NON spam'. Poi si stabilizza con l'uso reale.</t>
         </is>
       </c>
     </row>
@@ -734,22 +734,22 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Vortix / Lead</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Verificare che l'email di conferma arrivi al cliente</t>
+          <t>Cancellare il vecchio repository su GitHub</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Se il mittente non e' autorizzato sull'account Resend di Vortix, l'email al cliente non parte (in silenzio). La notifica interna a voi funziona comunque.</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Media</t>
+          <t>Il codice era stato caricato per errore sull'account personale calciolevelup-ai prima di creare quello aziendale. E' privato, quindi non e' urgente, ma va tolto.</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Bassa</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Fare una prenotazione di prova su greenmindgroup.pro/company con un'email VERA e controllare se arriva. Mittente usato: prenotazioni@greenmindgroup.pro</t>
+          <t>github.com/calciolevelup-ai/green-mind-group &gt; Settings &gt; Danger Zone &gt; Delete. La copia buona e' su greenmindgroupsrls.</t>
         </is>
       </c>
     </row>
@@ -779,17 +779,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Cancellare il vecchio repository su GitHub</t>
+          <t>Chiudere la falla di notify_root</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Il codice era stato caricato per errore sull'account personale calciolevelup-ai prima di creare quello aziendale. E' privato, quindi non e' urgente, ma va tolto.</t>
+          <t>Un utente registrato puo' inviare all'azienda un messaggio fingendo di essere un altro membro. Impatto basso (solo messaggi, nessun accesso a dati).</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -809,12 +809,12 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Michele</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>github.com/calciolevelup-ai/green-mind-group &gt; Settings &gt; Danger Zone &gt; Delete. La copia buona e' su greenmindgroupsrls.</t>
+          <t>Trovato nel controllo di sicurezza del 31/08. Correzione stimata: 5 minuti.</t>
         </is>
       </c>
     </row>
@@ -824,42 +824,42 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Piano compensi</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Chiudere la falla di notify_root</t>
+          <t>Decidere se allineare il piano compensi al modello CGI</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Un utente registrato puo' inviare all'azienda un messaggio fingendo di essere un altro membro. Impatto basso (solo messaggi, nessun accesso a dati).</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Bassa</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
+          <t>Il confronto col documento Casa Green Italy ha evidenziato 12 differenze, alcune importanti (pass-up, pagamento a cascata, finestra di recesso 14 giorni, tariffe ridotte con P.IVA).</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Bloccato</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>gratis</t>
+          <t>da valutare</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Michele</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Trovato nel controllo di sicurezza del 31/08. Correzione stimata: 5 minuti.</t>
+          <t>MESSO IN STANDBY dall'utente il 31/08. Vedi foglio 'Confronto CGI' per l'elenco completo delle differenze.</t>
         </is>
       </c>
     </row>
@@ -869,97 +869,52 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Piano compensi</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Decidere se allineare il piano compensi al modello CGI</t>
+          <t>Aggiungere indici sulle chiavi esterne mancanti</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Il confronto col documento Casa Green Italy ha evidenziato 12 differenze, alcune importanti (pass-up, pagamento a cascata, finestra di recesso 14 giorni, tariffe ridotte con P.IVA).</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Bloccato</t>
+          <t>12 segnalazioni informative su tabelle poco trafficate (audit log, eventi, documenti). Nessun impatto percepibile oggi.</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>da valutare</t>
+          <t>gratis</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Michele</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>MESSO IN STANDBY dall'utente il 31/08. Vedi foglio 'Confronto CGI' per l'elenco completo delle differenze.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Database</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Aggiungere indici sulle chiavi esterne mancanti</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>12 segnalazioni informative su tabelle poco trafficate (audit log, eventi, documenti). Nessun impatto percepibile oggi.</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>Bassa</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>gratis</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
           <t>Solo livello INFO nel controllo prestazioni Supabase. Da fare quando la rete cresce, non ora.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I12"/>
+  <autoFilter ref="A4:I11"/>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Da fare,In corso,Fatto,Bloccato"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Bassa"</formula1>
     </dataValidation>
   </dataValidations>
@@ -973,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1021,132 +976,132 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
+          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
+          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
+          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
+          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Controllo completo di sicurezza del database</t>
+          <t>Email di conferma migliorata contro lo spam</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
+          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
+          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
+          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
+          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Testato end-to-end con una prenotazione reale</t>
+          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
+          <t>Controllo completo di sicurezza del database</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
+          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
         </is>
       </c>
     </row>
@@ -1158,17 +1113,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
+          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
+          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
         </is>
       </c>
     </row>
@@ -1180,17 +1135,17 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Payout</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Prelievo bloccato se il profilo non e' completo</t>
+          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
+          <t>Testato end-to-end con una prenotazione reale</t>
         </is>
       </c>
     </row>
@@ -1202,17 +1157,17 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Mostra/nascondi password su tutti i campi password</t>
+          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
+          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1179,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Codice attivita' separato graficamente dall'username</t>
+          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Dashboard, albero, centro di controllo, contatti</t>
+          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
         </is>
       </c>
     </row>
@@ -1246,17 +1201,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Payout</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+          <t>Prelievo bloccato se il profilo non e' completo</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
         </is>
       </c>
     </row>
@@ -1268,17 +1223,17 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Centro controllo</t>
+          <t>Interfaccia</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Modifica username di un membro dall'account azienda</t>
+          <t>Mostra/nascondi password su tutti i campi password</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Con controllo anti-duplicato verificato sul database reale</t>
+          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
         </is>
       </c>
     </row>
@@ -1290,22 +1245,88 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Codice attivita' separato graficamente dall'username</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard, albero, centro di controllo, contatti</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Centro controllo</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Modifica username di un membro dall'account azienda</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Con controllo anti-duplicato verificato sul database reale</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
           <t>Affidabilita'</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Niente piu' dati finti in caso di errore di caricamento</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Prima, se il caricamento falliva, l'utente vedeva una rete inventata con l'avviso 'dati di esempio'</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D17"/>
+  <autoFilter ref="A4:D20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1367,7 +1388,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Prenotazione di prova su /company con email vera -&gt; arriva la conferma al cliente?</t>
+          <t>Ricontrollare tra qualche settimana se la conferma arriva in posta in arrivo (non spam)</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -1377,7 +1398,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>L'unico modo per chiudere la riga #4 di 'Da fare'</t>
+          <t>Serve la tua casella per verificarlo</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2064,27 +2085,49 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Il dominio e' nuovo e senza reputazione di invio</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Le email possono finire in spam finche' non si consolida lo storico di invio</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Segnalare 'non e' spam' e attendere: si stabilizza con l'uso reale</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>Generale</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Molte funzioni verificate solo sul database, non cliccate nel browser</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Il comportamento e' corretto, ma l'esperienza reale d'uso non e' mai stata provata</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Vedi foglio 'Da provare tu'</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D10"/>
+  <autoFilter ref="A4:D11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist: email VORTIX ridisegnata e font del sito verificati
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CHECKLIST.xlsx
+++ b/CHECKLIST.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Da provare tu'!$A$4:$D$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Confronto CGI'!$A$4:$E$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Limitazioni note'!$A$4:$D$11</definedName>
@@ -928,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -981,17 +981,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
+          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
+          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
         </is>
       </c>
     </row>
@@ -1008,12 +1008,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
+          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
+          <t>Erano resi con l'apostrofo invece che con l'accento</t>
         </is>
       </c>
     </row>
@@ -1030,41 +1030,41 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma migliorata contro lo spam</t>
+          <t>Notifica interna: mittente spostato sul dominio verificato</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
+          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
+          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
+          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1074,122 +1074,122 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
+          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
+          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Controllo completo di sicurezza del database</t>
+          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
+          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
+          <t>Email di conferma migliorata contro lo spam</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
+          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
+          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Testato end-to-end con una prenotazione reale</t>
+          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
+          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
+          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
+          <t>Controllo completo di sicurezza del database</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
+          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
         </is>
       </c>
     </row>
@@ -1201,17 +1201,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Payout</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Prelievo bloccato se il profilo non e' completo</t>
+          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
+          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
         </is>
       </c>
     </row>
@@ -1223,17 +1223,17 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Mostra/nascondi password su tutti i campi password</t>
+          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
+          <t>Testato end-to-end con una prenotazione reale</t>
         </is>
       </c>
     </row>
@@ -1245,17 +1245,17 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Codice attivita' separato graficamente dall'username</t>
+          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Dashboard, albero, centro di controllo, contatti</t>
+          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
         </is>
       </c>
     </row>
@@ -1267,17 +1267,17 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
         </is>
       </c>
     </row>
@@ -1289,17 +1289,17 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Centro controllo</t>
+          <t>Payout</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Modifica username di un membro dall'account azienda</t>
+          <t>Prelievo bloccato se il profilo non e' completo</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Con controllo anti-duplicato verificato sul database reale</t>
+          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
         </is>
       </c>
     </row>
@@ -1311,22 +1311,110 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Mostra/nascondi password su tutti i campi password</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Codice attivita' separato graficamente dall'username</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard, albero, centro di controllo, contatti</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Centro controllo</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Modifica username di un membro dall'account azienda</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Con controllo anti-duplicato verificato sul database reale</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
           <t>Affidabilita'</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>Niente piu' dati finti in caso di errore di caricamento</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Prima, se il caricamento falliva, l'utente vedeva una rete inventata con l'avviso 'dati di esempio'</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D20"/>
+  <autoFilter ref="A4:D24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Checklist: falla notify_root chiusa
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CHECKLIST.xlsx
+++ b/CHECKLIST.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limitazioni note" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Da provare tu'!$A$4:$D$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Confronto CGI'!$A$4:$E$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Limitazioni note'!$A$4:$D$11</definedName>
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -779,42 +779,42 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Piano compensi</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Chiudere la falla di notify_root</t>
+          <t>Decidere se allineare il piano compensi al modello CGI</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Un utente registrato puo' inviare all'azienda un messaggio fingendo di essere un altro membro. Impatto basso (solo messaggi, nessun accesso a dati).</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Bassa</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
+          <t>Il confronto col documento Casa Green Italy ha evidenziato 12 differenze, alcune importanti (pass-up, pagamento a cascata, finestra di recesso 14 giorni, tariffe ridotte con P.IVA).</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Bloccato</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>gratis</t>
+          <t>da valutare</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Michele</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Trovato nel controllo di sicurezza del 31/08. Correzione stimata: 5 minuti.</t>
+          <t>MESSO IN STANDBY dall'utente il 31/08. Vedi foglio 'Confronto CGI' per l'elenco completo delle differenze.</t>
         </is>
       </c>
     </row>
@@ -824,97 +824,52 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Piano compensi</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Decidere se allineare il piano compensi al modello CGI</t>
+          <t>Aggiungere indici sulle chiavi esterne mancanti</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Il confronto col documento Casa Green Italy ha evidenziato 12 differenze, alcune importanti (pass-up, pagamento a cascata, finestra di recesso 14 giorni, tariffe ridotte con P.IVA).</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Bloccato</t>
+          <t>12 segnalazioni informative su tabelle poco trafficate (audit log, eventi, documenti). Nessun impatto percepibile oggi.</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>da valutare</t>
+          <t>gratis</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Michele</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>MESSO IN STANDBY dall'utente il 31/08. Vedi foglio 'Confronto CGI' per l'elenco completo delle differenze.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Database</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Aggiungere indici sulle chiavi esterne mancanti</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>12 segnalazioni informative su tabelle poco trafficate (audit log, eventi, documenti). Nessun impatto percepibile oggi.</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>Bassa</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>gratis</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
           <t>Solo livello INFO nel controllo prestazioni Supabase. Da fare quando la rete cresce, non ora.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I11"/>
+  <autoFilter ref="A4:I10"/>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Da fare,In corso,Fatto,Bloccato"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Bassa"</formula1>
     </dataValidation>
   </dataValidations>
@@ -928,7 +883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -981,17 +936,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
+          <t>Chiusa la falsificazione del mittente in notify_root</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
+          <t>Doppia difesa: mittente letto dalla sessione reale + permesso revocato agli utenti. Verificato: chiamata diretta rifiutata, ticket di supporto continua a funzionare col mittente corretto</t>
         </is>
       </c>
     </row>
@@ -1008,12 +963,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
+          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Erano resi con l'apostrofo invece che con l'accento</t>
+          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
         </is>
       </c>
     </row>
@@ -1030,12 +985,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Notifica interna: mittente spostato sul dominio verificato</t>
+          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
+          <t>Erano resi con l'apostrofo invece che con l'accento</t>
         </is>
       </c>
     </row>
@@ -1047,17 +1002,17 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
+          <t>Notifica interna: mittente spostato sul dominio verificato</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
+          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
         </is>
       </c>
     </row>
@@ -1069,17 +1024,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
+          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
+          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
         </is>
       </c>
     </row>
@@ -1091,17 +1046,17 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
+          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
+          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
         </is>
       </c>
     </row>
@@ -1118,34 +1073,34 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma migliorata contro lo spam</t>
+          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
+          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
+          <t>Email di conferma migliorata contro lo spam</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
+          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
         </is>
       </c>
     </row>
@@ -1157,17 +1112,17 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
+          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
+          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
         </is>
       </c>
     </row>
@@ -1184,34 +1139,34 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Controllo completo di sicurezza del database</t>
+          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
+          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
+          <t>Controllo completo di sicurezza del database</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
+          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
         </is>
       </c>
     </row>
@@ -1228,12 +1183,12 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
+          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Testato end-to-end con una prenotazione reale</t>
+          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
         </is>
       </c>
     </row>
@@ -1245,17 +1200,17 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
+          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
+          <t>Testato end-to-end con una prenotazione reale</t>
         </is>
       </c>
     </row>
@@ -1267,17 +1222,17 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
+          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
+          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
         </is>
       </c>
     </row>
@@ -1289,17 +1244,17 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Payout</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Prelievo bloccato se il profilo non e' completo</t>
+          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
+          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
         </is>
       </c>
     </row>
@@ -1311,17 +1266,17 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Payout</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Mostra/nascondi password su tutti i campi password</t>
+          <t>Prelievo bloccato se il profilo non e' completo</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
+          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
         </is>
       </c>
     </row>
@@ -1338,12 +1293,12 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Codice attivita' separato graficamente dall'username</t>
+          <t>Mostra/nascondi password su tutti i campi password</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Dashboard, albero, centro di controllo, contatti</t>
+          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
         </is>
       </c>
     </row>
@@ -1360,12 +1315,12 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+          <t>Codice attivita' separato graficamente dall'username</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+          <t>Dashboard, albero, centro di controllo, contatti</t>
         </is>
       </c>
     </row>
@@ -1377,17 +1332,17 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Centro controllo</t>
+          <t>Interfaccia</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Modifica username di un membro dall'account azienda</t>
+          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Con controllo anti-duplicato verificato sul database reale</t>
+          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
         </is>
       </c>
     </row>
@@ -1399,22 +1354,44 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
+          <t>Centro controllo</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Modifica username di un membro dall'account azienda</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Con controllo anti-duplicato verificato sul database reale</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
           <t>Affidabilita'</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Niente piu' dati finti in caso di errore di caricamento</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Prima, se il caricamento falliva, l'utente vedeva una rete inventata con l'avviso 'dati di esempio'</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D24"/>
+  <autoFilter ref="A4:D25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Checklist: contratto incaricato fatto, aggiunta revisione legale
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CHECKLIST.xlsx
+++ b/CHECKLIST.xlsx
@@ -14,9 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limitazioni note" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Da provare tu'!$A$4:$D$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Da provare tu'!$A$4:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Confronto CGI'!$A$4:$E$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Limitazioni note'!$A$4:$D$11</definedName>
   </definedNames>
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -734,22 +734,22 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Legale</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Cancellare il vecchio repository su GitHub</t>
+          <t>Far revisionare da un legale il contratto incaricato firmato online</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Il codice era stato caricato per errore sull'account personale calciolevelup-ai prima di creare quello aziendale. E' privato, quindi non e' urgente, ma va tolto.</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>Bassa</t>
+          <t>L'art. 1341 c.c. richiede l'approvazione specifica PER ISCRITTO delle clausole onerose e la giurisprudenza e' severa sul valore della spunta online. Il sistema registra data, ora, IP e versione del testo per dare il massimo peso probatorio possibile, ma la validita' va confermata da un professionista.</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>gratis</t>
+          <t>da valutare</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>github.com/calciolevelup-ai/green-mind-group &gt; Settings &gt; Danger Zone &gt; Delete. La copia buona e' su greenmindgroupsrls.</t>
+          <t>Segnalato il 01/09 prima di costruire la funzione; l'azienda ha scelto consapevolmente l'accettazione interamente online. Se il legale lo richiede, si puo' aggiungere il passaggio 'stampa, firma a mano e ricarica'.</t>
         </is>
       </c>
     </row>
@@ -779,32 +779,32 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Piano compensi</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Decidere se allineare il piano compensi al modello CGI</t>
+          <t>Cancellare il vecchio repository su GitHub</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Il confronto col documento Casa Green Italy ha evidenziato 12 differenze, alcune importanti (pass-up, pagamento a cascata, finestra di recesso 14 giorni, tariffe ridotte con P.IVA).</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Bloccato</t>
+          <t>Il codice era stato caricato per errore sull'account personale calciolevelup-ai prima di creare quello aziendale. E' privato, quindi non e' urgente, ma va tolto.</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>da valutare</t>
+          <t>gratis</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>MESSO IN STANDBY dall'utente il 31/08. Vedi foglio 'Confronto CGI' per l'elenco completo delle differenze.</t>
+          <t>github.com/calciolevelup-ai/green-mind-group &gt; Settings &gt; Danger Zone &gt; Delete. La copia buona e' su greenmindgroupsrls.</t>
         </is>
       </c>
     </row>
@@ -824,52 +824,97 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>Piano compensi</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Decidere se allineare il piano compensi al modello CGI</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Il confronto col documento Casa Green Italy ha evidenziato 12 differenze, alcune importanti (pass-up, pagamento a cascata, finestra di recesso 14 giorni, tariffe ridotte con P.IVA).</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Bloccato</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>da valutare</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Michele</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>MESSO IN STANDBY dall'utente il 31/08. Vedi foglio 'Confronto CGI' per l'elenco completo delle differenze.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
           <t>Database</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Aggiungere indici sulle chiavi esterne mancanti</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>12 segnalazioni informative su tabelle poco trafficate (audit log, eventi, documenti). Nessun impatto percepibile oggi.</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>Bassa</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Da fare</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>gratis</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Solo livello INFO nel controllo prestazioni Supabase. Da fare quando la rete cresce, non ora.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I10"/>
+  <autoFilter ref="A4:I11"/>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Da fare,In corso,Fatto,Bloccato"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Bassa"</formula1>
     </dataValidation>
   </dataValidations>
@@ -883,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -936,17 +981,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Contratti</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Chiusa la falsificazione del mittente in notify_root</t>
+          <t>Contratto incaricato: form + generazione PDF + firma con spunte</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Doppia difesa: mittente letto dalla sessione reale + permesso revocato agli utenti. Verificato: chiamata diretta rifiutata, ticket di supporto continua a funzionare col mittente corretto</t>
+          <t>Verificato sul database: firma completa, doppia firma rifiutata, campi obbligatori validati. PDF generato e ispezionato: 5 pagine (dati + contratto originale integrale), accenti corretti</t>
         </is>
       </c>
     </row>
@@ -958,17 +1003,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
+          <t>Chiusa la falsificazione del mittente in notify_root</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
+          <t>Doppia difesa: mittente letto dalla sessione reale + permesso revocato agli utenti. Verificato: chiamata diretta rifiutata, ticket di supporto continua a funzionare col mittente corretto</t>
         </is>
       </c>
     </row>
@@ -985,12 +1030,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
+          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Erano resi con l'apostrofo invece che con l'accento</t>
+          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
         </is>
       </c>
     </row>
@@ -1007,12 +1052,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Notifica interna: mittente spostato sul dominio verificato</t>
+          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
+          <t>Erano resi con l'apostrofo invece che con l'accento</t>
         </is>
       </c>
     </row>
@@ -1024,17 +1069,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
+          <t>Notifica interna: mittente spostato sul dominio verificato</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
+          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
         </is>
       </c>
     </row>
@@ -1046,17 +1091,17 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
+          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
+          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
         </is>
       </c>
     </row>
@@ -1068,17 +1113,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
+          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
+          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
         </is>
       </c>
     </row>
@@ -1095,34 +1140,34 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma migliorata contro lo spam</t>
+          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
+          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
+          <t>Email di conferma migliorata contro lo spam</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
+          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
         </is>
       </c>
     </row>
@@ -1134,17 +1179,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
+          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
+          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
         </is>
       </c>
     </row>
@@ -1161,34 +1206,34 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Controllo completo di sicurezza del database</t>
+          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
+          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
+          <t>Controllo completo di sicurezza del database</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
+          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
         </is>
       </c>
     </row>
@@ -1205,12 +1250,12 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
+          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Testato end-to-end con una prenotazione reale</t>
+          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
         </is>
       </c>
     </row>
@@ -1222,17 +1267,17 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
+          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
+          <t>Testato end-to-end con una prenotazione reale</t>
         </is>
       </c>
     </row>
@@ -1244,17 +1289,17 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
+          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
+          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
         </is>
       </c>
     </row>
@@ -1266,17 +1311,17 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Payout</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Prelievo bloccato se il profilo non e' completo</t>
+          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
+          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
         </is>
       </c>
     </row>
@@ -1288,17 +1333,17 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Payout</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Mostra/nascondi password su tutti i campi password</t>
+          <t>Prelievo bloccato se il profilo non e' completo</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
+          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
         </is>
       </c>
     </row>
@@ -1315,12 +1360,12 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Codice attivita' separato graficamente dall'username</t>
+          <t>Mostra/nascondi password su tutti i campi password</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Dashboard, albero, centro di controllo, contatti</t>
+          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
         </is>
       </c>
     </row>
@@ -1337,12 +1382,12 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+          <t>Codice attivita' separato graficamente dall'username</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+          <t>Dashboard, albero, centro di controllo, contatti</t>
         </is>
       </c>
     </row>
@@ -1354,17 +1399,17 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Centro controllo</t>
+          <t>Interfaccia</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Modifica username di un membro dall'account azienda</t>
+          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Con controllo anti-duplicato verificato sul database reale</t>
+          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
         </is>
       </c>
     </row>
@@ -1376,22 +1421,44 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
+          <t>Centro controllo</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Modifica username di un membro dall'account azienda</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Con controllo anti-duplicato verificato sul database reale</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
           <t>Affidabilita'</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>Niente piu' dati finti in caso di errore di caricamento</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>Prima, se il caricamento falliva, l'utente vedeva una rete inventata con l'avviso 'dati di esempio'</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D25"/>
+  <autoFilter ref="A4:D26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1402,7 +1469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1473,7 +1540,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Inoltrare un lead a un incaricato -&gt; gli arriva la notifica nel back office?</t>
+          <t>Firmare il contratto incaricato da un account cliente vero (form, anteprima PDF, spunte)</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1483,7 +1550,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Serve un account incaricato vero per controllare</t>
+          <t>Serve un account cliente non ancora incaricato: non posso accedere io</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1560,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Richiesta di prelievo con profilo incompleto -&gt; viene bloccata?</t>
+          <t>Inoltrare un lead a un incaricato -&gt; gli arriva la notifica nel back office?</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -1503,7 +1570,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Verificato sul database, mai cliccato da una sessione reale</t>
+          <t>Serve un account incaricato vero per controllare</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1580,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Cambio password dalle impostazioni con il nuovo occhio mostra/nascondi</t>
+          <t>Richiesta di prelievo con profilo incompleto -&gt; viene bloccata?</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1523,7 +1590,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Richiede accesso reale, non posso provarlo io</t>
+          <t>Verificato sul database, mai cliccato da una sessione reale</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1600,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Iscrizione di un nuovo membro dal back office (pagina Registrazione)</t>
+          <t>Cambio password dalle impostazioni con il nuovo occhio mostra/nascondi</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1543,7 +1610,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Richiede accesso reale come incaricato</t>
+          <t>Richiede accesso reale, non posso provarlo io</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1620,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Modifica username di un membro dal Centro di controllo</t>
+          <t>Iscrizione di un nuovo membro dal back office (pagina Registrazione)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1563,7 +1630,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Verificato sul database, mai cliccato nel browser</t>
+          <t>Richiede accesso reale come incaricato</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1640,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Campanella notifiche: nuovo iscritto / nuova commissione</t>
+          <t>Modifica username di un membro dal Centro di controllo</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1583,7 +1650,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Provato solo con dati vuoti e test sul database</t>
+          <t>Verificato sul database, mai cliccato nel browser</t>
         </is>
       </c>
     </row>
@@ -1593,24 +1660,44 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>Campanella notifiche: nuovo iscritto / nuova commissione</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Provato solo con dati vuoti e test sul database</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>Email reali: ticket, referral, ordine, prelievo (contenuto e grafica)</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Da fare</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>L'invio funziona, i singoli contenuti non sono mai stati letti in una casella vera</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D12"/>
+  <autoFilter ref="A4:D13"/>
   <dataValidations count="1">
-    <dataValidation sqref="C5:C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Da fare,In corso,Fatto,Bloccato"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Checklist: chiuse le voci del 01/09
Pubblicazione automatica collegata, deploy sbloccati, identita' dei
salvataggi corretta, repository personale cancellato, contratto firmabile
anche dagli incaricati gia' attivi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CHECKLIST.xlsx
+++ b/CHECKLIST.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limitazioni note" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Da provare tu'!$A$4:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Confronto CGI'!$A$4:$E$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Limitazioni note'!$A$4:$D$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Limitazioni note'!$A$4:$D$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -542,7 +542,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Aggiornato al 1 settembre 2026. Usa i menu a tendina nelle colonne Priorita' e Stato per aggiornare la checklist.</t>
+          <t>Aggiornato al 1 settembre 2026 (pomeriggio). Usa i menu a tendina nelle colonne Priorita' e Stato per aggiornare la checklist.</t>
         </is>
       </c>
     </row>
@@ -779,32 +779,32 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Piano compensi</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Cancellare il vecchio repository su GitHub</t>
+          <t>Decidere se allineare il piano compensi al modello CGI</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Il codice era stato caricato per errore sull'account personale calciolevelup-ai prima di creare quello aziendale. E' privato, quindi non e' urgente, ma va tolto.</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Bassa</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
+          <t>Il confronto col documento Casa Green Italy ha evidenziato 12 differenze, alcune importanti (pass-up, pagamento a cascata, finestra di recesso 14 giorni, tariffe ridotte con P.IVA).</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Bloccato</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>gratis</t>
+          <t>da valutare</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>github.com/calciolevelup-ai/green-mind-group &gt; Settings &gt; Danger Zone &gt; Delete. La copia buona e' su greenmindgroupsrls.</t>
+          <t>MESSO IN STANDBY dall'utente il 31/08. Vedi foglio 'Confronto CGI' per l'elenco completo delle differenze.</t>
         </is>
       </c>
     </row>
@@ -824,97 +824,52 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Piano compensi</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Decidere se allineare il piano compensi al modello CGI</t>
+          <t>Aggiungere indici sulle chiavi esterne mancanti</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Il confronto col documento Casa Green Italy ha evidenziato 12 differenze, alcune importanti (pass-up, pagamento a cascata, finestra di recesso 14 giorni, tariffe ridotte con P.IVA).</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Bloccato</t>
+          <t>12 segnalazioni informative su tabelle poco trafficate (audit log, eventi, documenti). Nessun impatto percepibile oggi.</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>da valutare</t>
+          <t>gratis</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Michele</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>MESSO IN STANDBY dall'utente il 31/08. Vedi foglio 'Confronto CGI' per l'elenco completo delle differenze.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Database</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Aggiungere indici sulle chiavi esterne mancanti</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>12 segnalazioni informative su tabelle poco trafficate (audit log, eventi, documenti). Nessun impatto percepibile oggi.</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>Bassa</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>gratis</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
           <t>Solo livello INFO nel controllo prestazioni Supabase. Da fare quando la rete cresce, non ora.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I11"/>
+  <autoFilter ref="A4:I10"/>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Da fare,In corso,Fatto,Bloccato"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Bassa"</formula1>
     </dataValidation>
   </dataValidations>
@@ -928,7 +883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1003,17 +958,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Infrastruttura</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Chiusa la falsificazione del mittente in notify_root</t>
+          <t>Pubblicazione automatica: GitHub collegato a Vercel</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Doppia difesa: mittente letto dalla sessione reale + permesso revocato agli utenti. Verificato: chiamata diretta rifiutata, ticket di supporto continua a funzionare col mittente corretto</t>
+          <t>Provato sul campo: inviato un salvataggio SENZA lanciare comandi, la pubblicazione e' partita da sola e si e' conclusa in 43 secondi</t>
         </is>
       </c>
     </row>
@@ -1025,17 +980,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Infrastruttura</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
+          <t>Sbloccate le pubblicazioni (erano ferme da un'ora)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
+          <t>Il piano gratuito consente una compilazione per volta: i deploy accumulati bloccavano i successivi. Rimossi + corretta l'identita' dei salvataggi</t>
         </is>
       </c>
     </row>
@@ -1047,17 +1002,17 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
+          <t>Identita' dei salvataggi corretta da personale ad aziendale</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Erano resi con l'apostrofo invece che con l'accento</t>
+          <t>Firmavano 'calciolevelup-ai' anche sul repository aziendale; ora 'greenmindgroupsrls'</t>
         </is>
       </c>
     </row>
@@ -1069,17 +1024,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Notifica interna: mittente spostato sul dominio verificato</t>
+          <t>Cancellato il repository sull'account personale</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
+          <t>Verificato prima che quello aziendale fosse completo e allineato</t>
         </is>
       </c>
     </row>
@@ -1091,17 +1046,17 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Contratti</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
+          <t>Contratto firmabile anche dagli incaricati gia' attivi</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
+          <t>Prima venivano rimandati alla dashboard: il discrimine ora e' il contratto, non il ruolo. Aggiunto avviso in dashboard, altrimenti non l'avrebbero mai trovato</t>
         </is>
       </c>
     </row>
@@ -1118,12 +1073,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
+          <t>Chiusa la falsificazione del mittente in notify_root</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
+          <t>Doppia difesa: mittente letto dalla sessione reale + permesso revocato agli utenti. Verificato: chiamata diretta rifiutata, ticket di supporto continua a funzionare col mittente corretto</t>
         </is>
       </c>
     </row>
@@ -1140,12 +1095,12 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
+          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
+          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
         </is>
       </c>
     </row>
@@ -1162,63 +1117,63 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma migliorata contro lo spam</t>
+          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
+          <t>Erano resi con l'apostrofo invece che con l'accento</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
+          <t>Notifica interna: mittente spostato sul dominio verificato</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
+          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
+          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
+          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1228,122 +1183,122 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Controllo completo di sicurezza del database</t>
+          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
+          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
+          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
+          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
+          <t>Email di conferma migliorata contro lo spam</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Testato end-to-end con una prenotazione reale</t>
+          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
+          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
+          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
+          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
+          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Payout</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Prelievo bloccato se il profilo non e' completo</t>
+          <t>Controllo completo di sicurezza del database</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
+          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
         </is>
       </c>
     </row>
@@ -1355,17 +1310,17 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Mostra/nascondi password su tutti i campi password</t>
+          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
+          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
         </is>
       </c>
     </row>
@@ -1377,17 +1332,17 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Codice attivita' separato graficamente dall'username</t>
+          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Dashboard, albero, centro di controllo, contatti</t>
+          <t>Testato end-to-end con una prenotazione reale</t>
         </is>
       </c>
     </row>
@@ -1399,17 +1354,17 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
         </is>
       </c>
     </row>
@@ -1421,17 +1376,17 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Centro controllo</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Modifica username di un membro dall'account azienda</t>
+          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Con controllo anti-duplicato verificato sul database reale</t>
+          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
         </is>
       </c>
     </row>
@@ -1443,22 +1398,132 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
+          <t>Payout</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Prelievo bloccato se il profilo non e' completo</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Mostra/nascondi password su tutti i campi password</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Codice attivita' separato graficamente dall'username</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard, albero, centro di controllo, contatti</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Centro controllo</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Modifica username di un membro dall'account azienda</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Con controllo anti-duplicato verificato sul database reale</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
           <t>Affidabilita'</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Niente piu' dati finti in caso di errore di caricamento</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>Prima, se il caricamento falliva, l'utente vedeva una rete inventata con l'avviso 'dati di esempio'</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D26"/>
+  <autoFilter ref="A4:D31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2079,7 +2144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2237,49 +2302,71 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Vercel gratuito</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Il dominio e' nuovo e senza reputazione di invio</t>
+          <t>Una sola compilazione per volta</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Le email possono finire in spam finche' non si consolida lo storico di invio</t>
+          <t>Se si lanciano piu' pubblicazioni ravvicinate si incastrano e vengono bloccate: e' successo il 01/09, sito fermo per un'ora sulla versione precedente</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Segnalare 'non e' spam' e attendere: si stabilizza con l'uso reale</t>
+          <t>Risolto collegando GitHub: ora le pubblicazioni partono una alla volta in automatico</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Il dominio e' nuovo e senza reputazione di invio</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Le email possono finire in spam finche' non si consolida lo storico di invio</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Segnalare 'non e' spam' e attendere: si stabilizza con l'uso reale</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
           <t>Generale</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Molte funzioni verificate solo sul database, non cliccate nel browser</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Il comportamento e' corretto, ma l'esperienza reale d'uso non e' mai stata provata</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Vedi foglio 'Da provare tu'</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D11"/>
+  <autoFilter ref="A4:D12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Checklist: risolto lo spam delle email (10/10 su mail-tester)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CHECKLIST.xlsx
+++ b/CHECKLIST.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Limitazioni note" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Da provare tu'!$A$4:$D$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Confronto CGI'!$A$4:$E$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Limitazioni note'!$A$4:$D$12</definedName>
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -542,7 +542,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Aggiornato al 1 settembre 2026 (pomeriggio). Usa i menu a tendina nelle colonne Priorita' e Stato per aggiornare la checklist.</t>
+          <t>Aggiornato al 1 settembre 2026 (sera). Usa i menu a tendina nelle colonne Priorita' e Stato per aggiornare la checklist.</t>
         </is>
       </c>
     </row>
@@ -689,42 +689,42 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Vortix / Lead</t>
+          <t>Legale</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>L'email di conferma al cliente finisce nello spam</t>
+          <t>Far revisionare da un legale il contratto incaricato firmato online</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Il cliente riceve la conferma nella cartella spam invece che in posta in arrivo. Rischio concreto: molti non la vedono e pensano che la richiesta non sia arrivata.</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>In corso</t>
+          <t>L'art. 1341 c.c. richiede l'approvazione specifica PER ISCRITTO delle clausole onerose e la giurisprudenza e' severa sul valore della spunta online. Il sistema registra data, ora, IP e versione del testo per dare il massimo peso probatorio possibile, ma la validita' va confermata da un professionista.</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>gratis</t>
+          <t>da valutare</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Michele + Claude</t>
+          <t>Michele</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>01/09: verificato che SPF, DKIM, DMARC e percorso di ritorno sono TUTTI corretti. La causa e' la reputazione: il dominio e' nato il 26/08 e non ha ancora storico di invio. Migliorata l'email (versione testo, Reply-To, firma aziendale). AZIONE PER TE: apri l'email nello spam e premi 'Segnala come NON spam'. Poi si stabilizza con l'uso reale.</t>
+          <t>Segnalato il 01/09 prima di costruire la funzione; l'azienda ha scelto consapevolmente l'accettazione interamente online. Se il legale lo richiede, si puo' aggiungere il passaggio 'stampa, firma a mano e ricarica'.</t>
         </is>
       </c>
     </row>
@@ -734,27 +734,27 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Legale</t>
+          <t>Piano compensi</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Far revisionare da un legale il contratto incaricato firmato online</t>
+          <t>Decidere se allineare il piano compensi al modello CGI</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>L'art. 1341 c.c. richiede l'approvazione specifica PER ISCRITTO delle clausole onerose e la giurisprudenza e' severa sul valore della spunta online. Il sistema registra data, ora, IP e versione del testo per dare il massimo peso probatorio possibile, ma la validita' va confermata da un professionista.</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
+          <t>Il confronto col documento Casa Green Italy ha evidenziato 12 differenze, alcune importanti (pass-up, pagamento a cascata, finestra di recesso 14 giorni, tariffe ridotte con P.IVA).</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Bloccato</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Segnalato il 01/09 prima di costruire la funzione; l'azienda ha scelto consapevolmente l'accettazione interamente online. Se il legale lo richiede, si puo' aggiungere il passaggio 'stampa, firma a mano e ricarica'.</t>
+          <t>MESSO IN STANDBY dall'utente il 31/08. Vedi foglio 'Confronto CGI' per l'elenco completo delle differenze.</t>
         </is>
       </c>
     </row>
@@ -779,97 +779,52 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Piano compensi</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Decidere se allineare il piano compensi al modello CGI</t>
+          <t>Aggiungere indici sulle chiavi esterne mancanti</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Il confronto col documento Casa Green Italy ha evidenziato 12 differenze, alcune importanti (pass-up, pagamento a cascata, finestra di recesso 14 giorni, tariffe ridotte con P.IVA).</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Bloccato</t>
+          <t>12 segnalazioni informative su tabelle poco trafficate (audit log, eventi, documenti). Nessun impatto percepibile oggi.</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Bassa</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>da valutare</t>
+          <t>gratis</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Michele</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>MESSO IN STANDBY dall'utente il 31/08. Vedi foglio 'Confronto CGI' per l'elenco completo delle differenze.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Database</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Aggiungere indici sulle chiavi esterne mancanti</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>12 segnalazioni informative su tabelle poco trafficate (audit log, eventi, documenti). Nessun impatto percepibile oggi.</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>Bassa</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>gratis</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
           <t>Solo livello INFO nel controllo prestazioni Supabase. Da fare quando la rete cresce, non ora.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I10"/>
+  <autoFilter ref="A4:I9"/>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F5:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Da fare,In corso,Fatto,Bloccato"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Bassa"</formula1>
     </dataValidation>
   </dataValidations>
@@ -883,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -958,17 +913,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Infrastruttura</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Pubblicazione automatica: GitHub collegato a Vercel</t>
+          <t>Punteggio antispam da 7,5 a 10/10 su mail-tester</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Provato sul campo: inviato un salvataggio SENZA lanciare comandi, la pubblicazione e' partita da sola e si e' conclusa in 43 secondi</t>
+          <t>Test reali con prenotazioni vere prima e dopo la correzione</t>
         </is>
       </c>
     </row>
@@ -980,17 +935,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Infrastruttura</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Sbloccate le pubblicazioni (erano ferme da un'ora)</t>
+          <t>Corretto il mittente: era lo schema classico del phishing</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Il piano gratuito consente una compilazione per volta: i deploy accumulati bloccavano i successivi. Rimossi + corretta l'identita' dei salvataggi</t>
+          <t>From su dominio aziendale ma Reply-To su Gmail (FREEMAIL_FORGED_REPLYTO, -2,5 punti). Introdotto da Claude il 01/09 e corretto lo stesso giorno. Ora mittente unico: hello@greenmindgroup.pro, nessun Reply-To</t>
         </is>
       </c>
     </row>
@@ -1002,17 +957,17 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Identita' dei salvataggi corretta da personale ad aziendale</t>
+          <t>Filtro Gmail: le prenotazioni non finiscono piu' nello spam</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Firmavano 'calciolevelup-ai' anche sul repository aziendale; ora 'greenmindgroupsrls'</t>
+          <t>Impostato da Michele. Garantisce di non perdere lead a prescindere dalla reputazione del dominio</t>
         </is>
       </c>
     </row>
@@ -1024,17 +979,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Infrastruttura</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Cancellato il repository sull'account personale</t>
+          <t>Pubblicazione automatica: GitHub collegato a Vercel</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Verificato prima che quello aziendale fosse completo e allineato</t>
+          <t>Provato sul campo: inviato un salvataggio SENZA lanciare comandi, la pubblicazione e' partita da sola e si e' conclusa in 43 secondi</t>
         </is>
       </c>
     </row>
@@ -1046,17 +1001,17 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Contratti</t>
+          <t>Infrastruttura</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Contratto firmabile anche dagli incaricati gia' attivi</t>
+          <t>Sbloccate le pubblicazioni (erano ferme da un'ora)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Prima venivano rimandati alla dashboard: il discrimine ora e' il contratto, non il ruolo. Aggiunto avviso in dashboard, altrimenti non l'avrebbero mai trovato</t>
+          <t>Il piano gratuito consente una compilazione per volta: i deploy accumulati bloccavano i successivi. Rimossi + corretta l'identita' dei salvataggi</t>
         </is>
       </c>
     </row>
@@ -1068,17 +1023,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Chiusa la falsificazione del mittente in notify_root</t>
+          <t>Identita' dei salvataggi corretta da personale ad aziendale</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Doppia difesa: mittente letto dalla sessione reale + permesso revocato agli utenti. Verificato: chiamata diretta rifiutata, ticket di supporto continua a funzionare col mittente corretto</t>
+          <t>Firmavano 'calciolevelup-ai' anche sul repository aziendale; ora 'greenmindgroupsrls'</t>
         </is>
       </c>
     </row>
@@ -1090,17 +1045,17 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
+          <t>Cancellato il repository sull'account personale</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
+          <t>Verificato prima che quello aziendale fosse completo e allineato</t>
         </is>
       </c>
     </row>
@@ -1112,17 +1067,17 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Contratti</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
+          <t>Contratto firmabile anche dagli incaricati gia' attivi</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Erano resi con l'apostrofo invece che con l'accento</t>
+          <t>Prima venivano rimandati alla dashboard: il discrimine ora e' il contratto, non il ruolo. Aggiunto avviso in dashboard, altrimenti non l'avrebbero mai trovato</t>
         </is>
       </c>
     </row>
@@ -1134,17 +1089,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Notifica interna: mittente spostato sul dominio verificato</t>
+          <t>Chiusa la falsificazione del mittente in notify_root</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
+          <t>Doppia difesa: mittente letto dalla sessione reale + permesso revocato agli utenti. Verificato: chiamata diretta rifiutata, ticket di supporto continua a funzionare col mittente corretto</t>
         </is>
       </c>
     </row>
@@ -1156,17 +1111,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
+          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
+          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
         </is>
       </c>
     </row>
@@ -1178,17 +1133,17 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
+          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
+          <t>Erano resi con l'apostrofo invece che con l'accento</t>
         </is>
       </c>
     </row>
@@ -1205,12 +1160,12 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
+          <t>Notifica interna: mittente spostato sul dominio verificato</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
+          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
         </is>
       </c>
     </row>
@@ -1222,149 +1177,149 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma migliorata contro lo spam</t>
+          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
+          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
+          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
+          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
+          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
+          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Controllo completo di sicurezza del database</t>
+          <t>Email di conferma migliorata contro lo spam</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
+          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
+          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
+          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
+          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Testato end-to-end con una prenotazione reale</t>
+          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
+          <t>Controllo completo di sicurezza del database</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
+          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
         </is>
       </c>
     </row>
@@ -1376,17 +1331,17 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
+          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
+          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
         </is>
       </c>
     </row>
@@ -1398,17 +1353,17 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Payout</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Prelievo bloccato se il profilo non e' completo</t>
+          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
+          <t>Testato end-to-end con una prenotazione reale</t>
         </is>
       </c>
     </row>
@@ -1420,17 +1375,17 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Mostra/nascondi password su tutti i campi password</t>
+          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
+          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
         </is>
       </c>
     </row>
@@ -1442,17 +1397,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Codice attivita' separato graficamente dall'username</t>
+          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Dashboard, albero, centro di controllo, contatti</t>
+          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
         </is>
       </c>
     </row>
@@ -1464,17 +1419,17 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Payout</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+          <t>Prelievo bloccato se il profilo non e' completo</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
         </is>
       </c>
     </row>
@@ -1486,17 +1441,17 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Centro controllo</t>
+          <t>Interfaccia</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Modifica username di un membro dall'account azienda</t>
+          <t>Mostra/nascondi password su tutti i campi password</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Con controllo anti-duplicato verificato sul database reale</t>
+          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
         </is>
       </c>
     </row>
@@ -1508,22 +1463,88 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Codice attivita' separato graficamente dall'username</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard, albero, centro di controllo, contatti</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Centro controllo</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Modifica username di un membro dall'account azienda</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Con controllo anti-duplicato verificato sul database reale</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
           <t>Affidabilita'</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>Niente piu' dati finti in caso di errore di caricamento</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>Prima, se il caricamento falliva, l'utente vedeva una rete inventata con l'avviso 'dati di esempio'</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D31"/>
+  <autoFilter ref="A4:D34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2334,12 +2355,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Le email possono finire in spam finche' non si consolida lo storico di invio</t>
+          <t>Lato tecnico ora e' perfetto (10/10 su mail-tester), ma Gmail puo' ancora essere prudente coi mittenti nati da poco: qualche email al cliente potrebbe finire in spam nelle prime settimane</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Segnalare 'non e' spam' e attendere: si stabilizza con l'uso reale</t>
+          <t>Si risolve da solo con l'uso reale. Per la casella aziendale c'e' gia' un filtro Gmail che lo impedisce</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Checklist: aggiunto il calendario appuntamenti
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CHECKLIST.xlsx
+++ b/CHECKLIST.xlsx
@@ -15,8 +15,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Da fare'!$A$4:$I$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Da provare tu'!$A$4:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fatto di recente'!$A$4:$D$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Da provare tu'!$A$4:$D$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Confronto CGI'!$A$4:$E$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Limitazioni note'!$A$4:$D$12</definedName>
   </definedNames>
@@ -838,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -913,17 +913,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Punteggio antispam da 7,5 a 10/10 su mail-tester</t>
+          <t>Calendario appuntamenti nella scheda Lead</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Test reali con prenotazioni vere prima e dopo la correzione</t>
+          <t>Vista mensile con colori per stato e dettaglio giornaliero. Verificato in locale con dati realistici, incluso lo spostamento di un appuntamento su un giorno diverso da quello richiesto</t>
         </is>
       </c>
     </row>
@@ -935,17 +935,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Corretto il mittente: era lo schema classico del phishing</t>
+          <t>Distinzione tra orario richiesto e appuntamento confermato</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>From su dominio aziendale ma Reply-To su Gmail (FREEMAIL_FORGED_REPLYTO, -2,5 punti). Introdotto da Claude il 01/09 e corretto lo stesso giorno. Ora mittente unico: hello@greenmindgroup.pro, nessun Reply-To</t>
+          <t>La data dal sito e' quella che chiede il cliente, ma si fissa al telefono entro 24h e spesso si sposta: senza questa distinzione il calendario sarebbe divergente dalla realta' dopo la prima chiamata</t>
         </is>
       </c>
     </row>
@@ -962,12 +962,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Filtro Gmail: le prenotazioni non finiscono piu' nello spam</t>
+          <t>Punteggio antispam da 7,5 a 10/10 su mail-tester</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Impostato da Michele. Garantisce di non perdere lead a prescindere dalla reputazione del dominio</t>
+          <t>Test reali con prenotazioni vere prima e dopo la correzione</t>
         </is>
       </c>
     </row>
@@ -979,17 +979,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Infrastruttura</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Pubblicazione automatica: GitHub collegato a Vercel</t>
+          <t>Corretto il mittente: era lo schema classico del phishing</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Provato sul campo: inviato un salvataggio SENZA lanciare comandi, la pubblicazione e' partita da sola e si e' conclusa in 43 secondi</t>
+          <t>From su dominio aziendale ma Reply-To su Gmail (FREEMAIL_FORGED_REPLYTO, -2,5 punti). Introdotto da Claude il 01/09 e corretto lo stesso giorno. Ora mittente unico: hello@greenmindgroup.pro, nessun Reply-To</t>
         </is>
       </c>
     </row>
@@ -1001,17 +1001,17 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Infrastruttura</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Sbloccate le pubblicazioni (erano ferme da un'ora)</t>
+          <t>Filtro Gmail: le prenotazioni non finiscono piu' nello spam</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Il piano gratuito consente una compilazione per volta: i deploy accumulati bloccavano i successivi. Rimossi + corretta l'identita' dei salvataggi</t>
+          <t>Impostato da Michele. Garantisce di non perdere lead a prescindere dalla reputazione del dominio</t>
         </is>
       </c>
     </row>
@@ -1023,17 +1023,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Infrastruttura</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Identita' dei salvataggi corretta da personale ad aziendale</t>
+          <t>Pubblicazione automatica: GitHub collegato a Vercel</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Firmavano 'calciolevelup-ai' anche sul repository aziendale; ora 'greenmindgroupsrls'</t>
+          <t>Provato sul campo: inviato un salvataggio SENZA lanciare comandi, la pubblicazione e' partita da sola e si e' conclusa in 43 secondi</t>
         </is>
       </c>
     </row>
@@ -1045,17 +1045,17 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Infrastruttura</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Cancellato il repository sull'account personale</t>
+          <t>Sbloccate le pubblicazioni (erano ferme da un'ora)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Verificato prima che quello aziendale fosse completo e allineato</t>
+          <t>Il piano gratuito consente una compilazione per volta: i deploy accumulati bloccavano i successivi. Rimossi + corretta l'identita' dei salvataggi</t>
         </is>
       </c>
     </row>
@@ -1067,17 +1067,17 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Contratti</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Contratto firmabile anche dagli incaricati gia' attivi</t>
+          <t>Identita' dei salvataggi corretta da personale ad aziendale</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Prima venivano rimandati alla dashboard: il discrimine ora e' il contratto, non il ruolo. Aggiunto avviso in dashboard, altrimenti non l'avrebbero mai trovato</t>
+          <t>Firmavano 'calciolevelup-ai' anche sul repository aziendale; ora 'greenmindgroupsrls'</t>
         </is>
       </c>
     </row>
@@ -1089,17 +1089,17 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Chiusa la falsificazione del mittente in notify_root</t>
+          <t>Cancellato il repository sull'account personale</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Doppia difesa: mittente letto dalla sessione reale + permesso revocato agli utenti. Verificato: chiamata diretta rifiutata, ticket di supporto continua a funzionare col mittente corretto</t>
+          <t>Verificato prima che quello aziendale fosse completo e allineato</t>
         </is>
       </c>
     </row>
@@ -1111,17 +1111,17 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Contratti</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
+          <t>Contratto firmabile anche dagli incaricati gia' attivi</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
+          <t>Prima venivano rimandati alla dashboard: il discrimine ora e' il contratto, non il ruolo. Aggiunto avviso in dashboard, altrimenti non l'avrebbero mai trovato</t>
         </is>
       </c>
     </row>
@@ -1133,17 +1133,17 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
+          <t>Chiusa la falsificazione del mittente in notify_root</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Erano resi con l'apostrofo invece che con l'accento</t>
+          <t>Doppia difesa: mittente letto dalla sessione reale + permesso revocato agli utenti. Verificato: chiamata diretta rifiutata, ticket di supporto continua a funzionare col mittente corretto</t>
         </is>
       </c>
     </row>
@@ -1160,12 +1160,12 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Notifica interna: mittente spostato sul dominio verificato</t>
+          <t>Email ridisegnata nei colori del brand VORTIX (teal, sabbia, oro)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
+          <t>Anteprima verificata nel browser su desktop e mobile. Prima usava per errore i colori verdi di Green Mind Group</t>
         </is>
       </c>
     </row>
@@ -1177,17 +1177,17 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
+          <t>Corretti gli accenti italiani nelle email (accenti corretti)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
+          <t>Erano resi con l'apostrofo invece che con l'accento</t>
         </is>
       </c>
     </row>
@@ -1199,17 +1199,17 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
+          <t>Notifica interna: mittente spostato sul dominio verificato</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
+          <t>Il mittente di prova di Resend poteva scrivere SOLO al titolare account; ora le notifiche possono andare a qualsiasi indirizzo</t>
         </is>
       </c>
     </row>
@@ -1221,17 +1221,17 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
+          <t>Verificati i font su /company: coerenti su tutte le pagine</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
+          <t>Controllo dal vivo nel browser: General Sans e JetBrains Mono caricati e applicati davvero (misurata la larghezza del testo disegnato)</t>
         </is>
       </c>
     </row>
@@ -1243,61 +1243,61 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma migliorata contro lo spam</t>
+          <t>Lunghezza minima password portata a 8 caratteri su Supabase</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
+          <t>Impostato da Michele nel pannello. Ora il controllo e' applicato dal server, non piu' solo dal browser</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
+          <t>Email di conferma al cliente: CONFERMATA funzionante</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
+          <t>Prenotazione di prova reale: l'email parte e arriva. Finisce pero' in spam - vedi riga #3 in 'Da fare'</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>31/08</t>
+          <t>01/09</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
+          <t>Email di conferma migliorata contro lo spam</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
+          <t>Aggiunta versione in testo semplice, Reply-To su casella reale, firma aziendale completa</t>
         </is>
       </c>
     </row>
@@ -1309,61 +1309,61 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Sicurezza</t>
+          <t>Codice</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Controllo completo di sicurezza del database</t>
+          <t>Repository privato su GitHub aziendale (greenmindgroupsrls)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
+          <t>Verificato: privato, 258 file, 50 migrazioni, nessuna chiave segreta caricata</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
+          <t>Limite tentativi di accesso (max 40/minuto per IP, blocco 15 min)</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
+          <t>Pubblicato e verificato in produzione. Il piano Vercel gratuito ne consente uno solo.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>28/08</t>
+          <t>31/08</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>Sicurezza</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
+          <t>Controllo completo di sicurezza del database</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Testato end-to-end con una prenotazione reale</t>
+          <t>42 funzioni sensibili verificate: tutte quelle riservate all'azienda hanno il controllo di autorizzazione corretto</t>
         </is>
       </c>
     </row>
@@ -1375,17 +1375,17 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Sito</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
+          <t>Colonna 'Inoltra' per assegnare un lead a un incaricato</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
+          <t>Chi riceve il lead ottiene una notifica nel back office con i dati del contatto</t>
         </is>
       </c>
     </row>
@@ -1397,17 +1397,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Vortix</t>
+          <t>Lead</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
+          <t>Scheda Lead in Marketing (solo azienda) collegata al sito Vortix</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
+          <t>Testato end-to-end con una prenotazione reale</t>
         </is>
       </c>
     </row>
@@ -1419,17 +1419,17 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Payout</t>
+          <t>Sito</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Prelievo bloccato se il profilo non e' completo</t>
+          <t>Sito Vortix pubblicato su greenmindgroup.pro/company</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
+          <t>Verificato: pagina, grafica e file di stile caricati correttamente</t>
         </is>
       </c>
     </row>
@@ -1441,17 +1441,17 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Vortix</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Mostra/nascondi password su tutti i campi password</t>
+          <t>Email di conferma prenotazione al cliente (entro 24h vi contatta un tecnico)</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
+          <t>ATTENZIONE: scritta e attivata ma mai vista partire davvero - vedi riga #4 in 'Da fare'</t>
         </is>
       </c>
     </row>
@@ -1463,17 +1463,17 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Interfaccia</t>
+          <t>Payout</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Codice attivita' separato graficamente dall'username</t>
+          <t>Prelievo bloccato se il profilo non e' completo</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Dashboard, albero, centro di controllo, contatti</t>
+          <t>Controllo applicato nel database, non aggirabile dall'interfaccia</t>
         </is>
       </c>
     </row>
@@ -1490,12 +1490,12 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+          <t>Mostra/nascondi password su tutti i campi password</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+          <t>5 schermate: accesso, registrazione, reset, cambio password, iscrizione da back office</t>
         </is>
       </c>
     </row>
@@ -1507,17 +1507,17 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Centro controllo</t>
+          <t>Interfaccia</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Modifica username di un membro dall'account azienda</t>
+          <t>Codice attivita' separato graficamente dall'username</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Con controllo anti-duplicato verificato sul database reale</t>
+          <t>Dashboard, albero, centro di controllo, contatti</t>
         </is>
       </c>
     </row>
@@ -1529,22 +1529,66 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Corretto il clic sui nodi dell'albero (non apriva il dettaglio)</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Il riquadro di trascinamento rubava il clic al pulsante</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Centro controllo</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Modifica username di un membro dall'account azienda</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Con controllo anti-duplicato verificato sul database reale</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>28/08</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
           <t>Affidabilita'</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Niente piu' dati finti in caso di errore di caricamento</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>Prima, se il caricamento falliva, l'utente vedeva una rete inventata con l'avviso 'dati di esempio'</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D34"/>
+  <autoFilter ref="A4:D36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1555,7 +1599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1646,7 +1690,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Inoltrare un lead a un incaricato -&gt; gli arriva la notifica nel back office?</t>
+          <t>Calendario Lead: fissare e spostare un appuntamento con un lead vero</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -1656,7 +1700,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Serve un account incaricato vero per controllare</t>
+          <t>Provato solo con dati di prova in locale: serve un lead reale dal sito</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1710,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Richiesta di prelievo con profilo incompleto -&gt; viene bloccata?</t>
+          <t>Inoltrare un lead a un incaricato -&gt; gli arriva la notifica nel back office?</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1676,7 +1720,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Verificato sul database, mai cliccato da una sessione reale</t>
+          <t>Serve un account incaricato vero per controllare</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1730,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Cambio password dalle impostazioni con il nuovo occhio mostra/nascondi</t>
+          <t>Richiesta di prelievo con profilo incompleto -&gt; viene bloccata?</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1696,7 +1740,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Richiede accesso reale, non posso provarlo io</t>
+          <t>Verificato sul database, mai cliccato da una sessione reale</t>
         </is>
       </c>
     </row>
@@ -1706,7 +1750,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Iscrizione di un nuovo membro dal back office (pagina Registrazione)</t>
+          <t>Cambio password dalle impostazioni con il nuovo occhio mostra/nascondi</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1716,7 +1760,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Richiede accesso reale come incaricato</t>
+          <t>Richiede accesso reale, non posso provarlo io</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1770,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Modifica username di un membro dal Centro di controllo</t>
+          <t>Iscrizione di un nuovo membro dal back office (pagina Registrazione)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1736,7 +1780,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Verificato sul database, mai cliccato nel browser</t>
+          <t>Richiede accesso reale come incaricato</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1790,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Campanella notifiche: nuovo iscritto / nuova commissione</t>
+          <t>Modifica username di un membro dal Centro di controllo</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1756,7 +1800,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Provato solo con dati vuoti e test sul database</t>
+          <t>Verificato sul database, mai cliccato nel browser</t>
         </is>
       </c>
     </row>
@@ -1766,24 +1810,44 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>Campanella notifiche: nuovo iscritto / nuova commissione</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Da fare</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Provato solo con dati vuoti e test sul database</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
           <t>Email reali: ticket, referral, ordine, prelievo (contenuto e grafica)</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Da fare</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>L'invio funziona, i singoli contenuti non sono mai stati letti in una casella vera</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D13"/>
+  <autoFilter ref="A4:D14"/>
   <dataValidations count="1">
-    <dataValidation sqref="C5:C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:C14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Da fare,In corso,Fatto,Bloccato"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Checklist: aggiunta la voce sulla traduzione da finire
Riga 6 nel foglio 'Da fare', stato In corso: menu, campanella e schermate
di accesso sono tradotti, restano circa 300 frasi su un centinaio di file.
Nelle note l'ordine proposto e i due blocchi da non tradurre senza un
legale (contratto incaricato, Termini e Privacy).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CHECKLIST.xlsx
+++ b/CHECKLIST.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -815,6 +815,53 @@
       <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Solo livello INFO nel controllo prestazioni Supabase. Da fare quando la rete cresce, non ora.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Interfaccia</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Finire la traduzione del back office</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Oggi sono tradotti solo il menu, la campanella e le schermate di accesso. Il resto resta in italiano: funziona, ma un incaricato straniero trova meta' sistema nella sua lingua e meta' no.</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>In corso</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>gratis</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>Restano circa 300 frasi (1.500 traduzioni su 5 lingue) su un centinaio di file. Ordine proposto: Dashboard/Impostazioni/Payout, poi Team/Registrazione/Shop/Messaggi/Support, poi Marketing/Eventi. Centro di controllo per ultimo (lo usa solo l'azienda). NON tradurre senza un legale: contratto incaricato, Termini, Privacy.</t>
         </is>
       </c>
     </row>

</xml_diff>